<commit_message>
ConfigureChangeAndRestoreAllParametersTest - Fully tested and working correctly
</commit_message>
<xml_diff>
--- a/Power GUI AU-Tests Master.xlsx
+++ b/Power GUI AU-Tests Master.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://redlertechnologies734-my.sharepoint.com/personal/qa_redlertechnologies_com/Documents/PowerAutomation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://redlertechnologies734-my.sharepoint.com/personal/chavy_redlertechnologies_com/Documents/QA/Power/scripts/PowerGUIAutomation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_96267F21559302C5F0B75957C2F61C99FEB4DF65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_96267F21559302C5F0B75957C2F61C99FEB4DF65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2B6A46F-4AB1-4889-9892-80CD800A6FE1}"/>
   <bookViews>
-    <workbookView xWindow="504" yWindow="300" windowWidth="21600" windowHeight="11292" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-225" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RD152 Parameters" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18687" uniqueCount="734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18685" uniqueCount="734">
   <si>
     <t>Channel</t>
   </si>
@@ -2334,7 +2334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2373,6 +2373,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2709,15 +2712,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E1048576"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" style="2" customWidth="1"/>
     <col min="2" max="2" width="38" style="1" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="47.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" style="3" customWidth="1"/>
-    <col min="6" max="8" width="9.109375" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="1"/>
+    <col min="6" max="8" width="9.140625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -16721,12 +16724,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E619"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="47.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16879,8 +16882,8 @@
       <c r="D9" t="s">
         <v>36</v>
       </c>
-      <c r="E9" t="s">
-        <v>37</v>
+      <c r="E9" s="15">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -27262,7 +27265,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E80"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="38" customWidth="1"/>
@@ -28639,7 +28642,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E823"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="38" customWidth="1"/>
@@ -42647,7 +42650,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E796"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="38" customWidth="1"/>
@@ -42804,8 +42807,8 @@
       <c r="D9" t="s">
         <v>36</v>
       </c>
-      <c r="E9" t="s">
-        <v>37</v>
+      <c r="E9" s="15">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -56196,7 +56199,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E823"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="38" customWidth="1"/>
@@ -70204,7 +70207,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E613"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="38" customWidth="1"/>
@@ -80642,25 +80645,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:Q28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="70.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="59.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="70.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">

</xml_diff>